<commit_message>
Updated Login Error Manual Test Case
</commit_message>
<xml_diff>
--- a/Q1_TestCases.xlsx
+++ b/Q1_TestCases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Playwright\ecommerce-automation-test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E51F3C97-E451-4319-A798-A285EDA68230}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{804DE9C4-0132-463E-A116-DAC594AAE949}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -132,20 +132,59 @@
     </r>
   </si>
   <si>
-    <t>Manual Test Case: Verify Locked Out User Login Error
-Application URL:
+    <r>
+      <rPr>
+        <b/>
+        <sz val="13"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Manual Test Case: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Verify Locked Out User Login Error
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="13"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Application URL:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
 SauceDemo
-Test Case ID
-TC_LOGIN_005
-Test Scenario
-Verify that a locked-out user cannot log in and receives the correct error message.</t>
+</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -165,6 +204,28 @@
       <b/>
       <sz val="11"/>
       <color rgb="FF00B050"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="13"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -190,7 +251,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -207,8 +268,11 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -490,7 +554,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.453125" customWidth="1"/>
@@ -503,94 +567,103 @@
     <col min="8" max="8" width="24.90625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="362.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="6" t="s">
+    <row r="1" spans="1:12" s="6" customFormat="1" ht="87" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6"/>
-      <c r="F1" s="6"/>
-      <c r="G1" s="6"/>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A3" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B3" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D3" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="F3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="G3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="H3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="I4" s="2" t="s">
+      <c r="I3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="J4" s="2" t="s">
+      <c r="J3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="K4" s="2" t="s">
+      <c r="K3" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="L4" s="2" t="s">
+      <c r="L3" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:12" s="3" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
-      <c r="A5" s="1" t="s">
+    <row r="4" spans="1:12" ht="130.5" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B4" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C4" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D4" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E4" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="F4" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="G4" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="H5" s="4" t="s">
+      <c r="H4" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="I5" s="5" t="s">
+      <c r="I4" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="J5" s="1" t="s">
+      <c r="J4" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="K5" s="1" t="s">
+      <c r="K4" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="L5" s="1"/>
+      <c r="L4" s="1"/>
+    </row>
+    <row r="15" spans="1:12" ht="14.5" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="16" spans="1:12" s="3" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A16"/>
+      <c r="B16"/>
+      <c r="C16"/>
+      <c r="D16"/>
+      <c r="E16"/>
+      <c r="F16"/>
+      <c r="G16"/>
+      <c r="H16"/>
+      <c r="I16"/>
+      <c r="J16"/>
+      <c r="K16"/>
+      <c r="L16"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A1:XFD1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>